<commit_message>
web programming stuff, first week
</commit_message>
<xml_diff>
--- a/stats for com eng/excel files/Ch07-01.xlsx
+++ b/stats for com eng/excel files/Ch07-01.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pin/Desktop/joint-repository/stats for com eng/excel files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4002827-FF6B-FE47-9DD3-D58843F289E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9A805D7-8FF5-C046-B51D-A9CA3D6AA6A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="20480" windowHeight="11040" activeTab="1" xr2:uid="{6CA4CF82-2607-4099-8656-DF6CD5F2B5F5}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="20480" windowHeight="11040" activeTab="2" xr2:uid="{6CA4CF82-2607-4099-8656-DF6CD5F2B5F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Thickness" sheetId="1" r:id="rId1"/>
     <sheet name="Wraping" sheetId="2" r:id="rId2"/>
+    <sheet name="Wraping practice" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="75">
   <si>
     <t>Treatment Combination</t>
   </si>
@@ -217,6 +218,51 @@
   </si>
   <si>
     <t>It is signifcant because it is below 0.05, because that is an alpha, significant value</t>
+  </si>
+  <si>
+    <t>effect estimator</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>standard error</t>
+  </si>
+  <si>
+    <t>sigma^2</t>
+  </si>
+  <si>
+    <t>standard eror</t>
+  </si>
+  <si>
+    <t>t ratio</t>
+  </si>
+  <si>
+    <t>P value</t>
+  </si>
+  <si>
+    <t>df</t>
+  </si>
+  <si>
+    <t>alpha</t>
+  </si>
+  <si>
+    <t>sig</t>
+  </si>
+  <si>
+    <t>Coef</t>
+  </si>
+  <si>
+    <t>y intercept</t>
+  </si>
+  <si>
+    <t>predictor</t>
+  </si>
+  <si>
+    <t>y=5.375*B+22</t>
   </si>
 </sst>
 </file>
@@ -388,7 +434,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -498,12 +544,63 @@
     <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="1" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -531,55 +628,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -975,6 +1024,194 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>672393</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>83256</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>580460</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>122167</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5BD471E-02F4-B549-9594-9499B4C36E30}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="9067093" y="337256"/>
+          <a:ext cx="6194567" cy="2070911"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>593018</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>89605</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>491823</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>221050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1F945B35-0EDE-5941-9D21-2D5F83B7CC87}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8987718" y="2629605"/>
+          <a:ext cx="6185305" cy="2290445"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>473729</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>86641</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>391321</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>135910</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5FB7E5C9-240F-7846-A999-E3EB5481D111}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8868429" y="5293641"/>
+          <a:ext cx="6204092" cy="2843269"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -1284,28 +1521,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="1" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="44" t="s">
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="45" t="s">
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="46"/>
-      <c r="K1" s="47"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="64"/>
     </row>
     <row r="2" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="43"/>
+      <c r="A2" s="60"/>
       <c r="B2" s="10" t="s">
         <v>2</v>
       </c>
@@ -1315,10 +1552,10 @@
       <c r="D2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
       <c r="I2" s="11" t="s">
         <v>6</v>
       </c>
@@ -1549,54 +1786,54 @@
       </c>
     </row>
     <row r="27" spans="7:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G27" s="37" t="s">
+      <c r="G27" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="H27" s="38"/>
-      <c r="I27" s="38"/>
+      <c r="H27" s="52"/>
+      <c r="I27" s="52"/>
       <c r="J27" s="14">
         <f>AVERAGE(K3:K6)</f>
         <v>2.0790041666666703E-2</v>
       </c>
     </row>
     <row r="28" spans="7:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G28" s="37" t="s">
+      <c r="G28" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="H28" s="38" t="s">
+      <c r="H28" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="I28" s="38"/>
+      <c r="I28" s="52"/>
       <c r="J28" s="21">
         <f>J27/(4*2^(2-2))</f>
         <v>5.1975104166666758E-3</v>
       </c>
-      <c r="K28" s="61" t="s">
+      <c r="K28" s="37" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="29" spans="7:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G29" s="37" t="s">
+      <c r="G29" s="55" t="s">
         <v>21</v>
       </c>
-      <c r="H29" s="38" t="s">
+      <c r="H29" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="I29" s="38"/>
+      <c r="I29" s="52"/>
       <c r="J29" s="21">
         <f>SQRT(J28)</f>
         <v>7.2093761288107835E-2</v>
       </c>
-      <c r="K29" s="61" t="s">
+      <c r="K29" s="37" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="30" spans="7:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G30" s="39" t="s">
+      <c r="G30" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="H30" s="40"/>
-      <c r="I30" s="41"/>
+      <c r="H30" s="57"/>
+      <c r="I30" s="58"/>
       <c r="J30" s="22">
         <f>2^(2)*(4-1)</f>
         <v>12</v>
@@ -1646,7 +1883,7 @@
         <f>_xlfn.T.DIST.2T(D46, 12)</f>
         <v>7.0759204989125005E-8</v>
       </c>
-      <c r="F46" s="62" t="s">
+      <c r="F46" s="38" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1695,46 +1932,46 @@
       <c r="F48" s="24"/>
     </row>
     <row r="50" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="38" t="s">
+      <c r="A50" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="B50" s="38"/>
+      <c r="B50" s="52"/>
       <c r="C50" s="9">
         <f>AVERAGE(E3:H6)</f>
         <v>14.388874999999999</v>
       </c>
-      <c r="D50" s="61" t="s">
+      <c r="D50" s="37" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="38" t="s">
+      <c r="A51" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="B51" s="49"/>
+      <c r="B51" s="54"/>
       <c r="C51" s="9">
         <f>B46/2</f>
         <v>0.41799999999999926</v>
       </c>
-      <c r="D51" s="61" t="s">
+      <c r="D51" s="37" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="38" t="s">
+      <c r="A52" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="B52" s="49"/>
+      <c r="B52" s="54"/>
       <c r="C52" s="9">
         <f>B47/2</f>
         <v>-3.362499999999935E-2</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="38" t="s">
+      <c r="A53" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="B53" s="49"/>
+      <c r="B53" s="54"/>
       <c r="C53" s="9">
         <f>B48/2</f>
         <v>1.5749999999999265E-2</v>
@@ -1746,17 +1983,17 @@
       </c>
     </row>
     <row r="55" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="38" t="s">
+      <c r="A55" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="B55" s="38"/>
-      <c r="C55" s="48" t="s">
+      <c r="B55" s="52"/>
+      <c r="C55" s="53" t="s">
         <v>51</v>
       </c>
-      <c r="D55" s="48"/>
-      <c r="E55" s="48"/>
-      <c r="F55" s="48"/>
-      <c r="G55" s="48"/>
+      <c r="D55" s="53"/>
+      <c r="E55" s="53"/>
+      <c r="F55" s="53"/>
+      <c r="G55" s="53"/>
       <c r="I55" s="6" t="s">
         <v>50</v>
       </c>
@@ -1775,7 +2012,7 @@
         <f>0.418 * (-1) + 14.389</f>
         <v>13.971</v>
       </c>
-      <c r="F57" s="63" t="s">
+      <c r="F57" s="39" t="s">
         <v>52</v>
       </c>
       <c r="H57" s="6" t="s">
@@ -1790,7 +2027,7 @@
         <v>39</v>
       </c>
       <c r="E58" s="6">
-        <f t="shared" ref="E58:E60" si="4">0.418 * (-1) + 14.389</f>
+        <f t="shared" ref="E58" si="4">0.418 * (-1) + 14.389</f>
         <v>13.971</v>
       </c>
     </row>
@@ -1820,12 +2057,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A55:B55"/>
-    <mergeCell ref="C55:G55"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A53:B53"/>
     <mergeCell ref="G27:I27"/>
     <mergeCell ref="G29:I29"/>
     <mergeCell ref="G30:I30"/>
@@ -1834,6 +2065,12 @@
     <mergeCell ref="E1:H2"/>
     <mergeCell ref="I1:K1"/>
     <mergeCell ref="G28:I28"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="C55:G55"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A53:B53"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1855,26 +2092,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="58" t="s">
+      <c r="B1" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="60" t="s">
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="60"/>
-      <c r="G1" s="50" t="s">
+      <c r="F1" s="51"/>
+      <c r="G1" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="H1" s="51"/>
-      <c r="I1" s="52"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
     </row>
     <row r="2" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="59"/>
+      <c r="A2" s="50"/>
       <c r="B2" s="26" t="s">
         <v>2</v>
       </c>
@@ -1884,8 +2121,8 @@
       <c r="D2" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
       <c r="G2" s="27" t="s">
         <v>6</v>
       </c>
@@ -2080,10 +2317,10 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="53" t="s">
+      <c r="A12" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="B12" s="54"/>
+      <c r="B12" s="45"/>
       <c r="C12" s="31">
         <f>AVERAGE(I3:I6)</f>
         <v>9.375</v>
@@ -2094,10 +2331,10 @@
       <c r="H12" s="5"/>
     </row>
     <row r="13" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="55" t="s">
+      <c r="A13" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="54"/>
+      <c r="B13" s="45"/>
       <c r="C13" s="32">
         <f>SQRT((C12)/(E8*2^(E9-2)))</f>
         <v>2.1650635094610968</v>
@@ -2108,10 +2345,10 @@
       <c r="H13" s="5"/>
     </row>
     <row r="14" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="53" t="s">
+      <c r="A14" s="44" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="54"/>
+      <c r="B14" s="45"/>
       <c r="C14" s="30">
         <f>2^E9*(E8-1)</f>
         <v>4</v>
@@ -2263,16 +2500,16 @@
       <c r="H25" s="5"/>
     </row>
     <row r="27" spans="1:9" s="6" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="56" t="s">
+      <c r="A27" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="B27" s="56"/>
-      <c r="C27" s="57" t="s">
+      <c r="B27" s="47"/>
+      <c r="C27" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="D27" s="57"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="57"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="48"/>
+      <c r="F27" s="48"/>
       <c r="H27" s="16"/>
       <c r="I27" s="5"/>
     </row>
@@ -2298,7 +2535,7 @@
       <c r="C30" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E30" s="64">
+      <c r="E30" s="40">
         <f xml:space="preserve"> 5.375 *( 1)+ 21.625</f>
         <v>27</v>
       </c>
@@ -2343,4 +2580,494 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C0F7CD6-71AD-B243-8768-B066B0B62215}">
+  <dimension ref="A1:K32"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="20.25" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.6640625" style="5" customWidth="1"/>
+    <col min="2" max="4" width="10.6640625" style="5" customWidth="1"/>
+    <col min="5" max="7" width="10.6640625" style="6" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="16" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" style="5" customWidth="1"/>
+    <col min="10" max="16384" width="9.1640625" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="1" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="49" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="51" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="51"/>
+      <c r="G1" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1" s="42"/>
+      <c r="I1" s="43"/>
+    </row>
+    <row r="2" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="50"/>
+      <c r="B2" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="25">
+        <v>17</v>
+      </c>
+      <c r="F3" s="25">
+        <v>20</v>
+      </c>
+      <c r="G3" s="30">
+        <f>SUM(E3:F3)</f>
+        <v>37</v>
+      </c>
+      <c r="H3" s="31">
+        <f>AVERAGE(E3:F3)</f>
+        <v>18.5</v>
+      </c>
+      <c r="I3" s="31">
+        <f>_xlfn.VAR.S(E3:F3)</f>
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="25">
+        <v>16</v>
+      </c>
+      <c r="F4" s="25">
+        <v>12</v>
+      </c>
+      <c r="G4" s="30">
+        <f t="shared" ref="G4:G6" si="0">SUM(E4:F4)</f>
+        <v>28</v>
+      </c>
+      <c r="H4" s="31">
+        <f t="shared" ref="H4:H6" si="1">AVERAGE(E4:F4)</f>
+        <v>14</v>
+      </c>
+      <c r="I4" s="31">
+        <f t="shared" ref="I4:I6" si="2">_xlfn.VAR.S(E4:F4)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="25">
+        <v>28</v>
+      </c>
+      <c r="F5" s="25">
+        <v>27</v>
+      </c>
+      <c r="G5" s="30">
+        <f t="shared" si="0"/>
+        <v>55</v>
+      </c>
+      <c r="H5" s="31">
+        <f t="shared" si="1"/>
+        <v>27.5</v>
+      </c>
+      <c r="I5" s="31">
+        <f t="shared" si="2"/>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="25">
+        <v>30</v>
+      </c>
+      <c r="F6" s="25">
+        <v>23</v>
+      </c>
+      <c r="G6" s="30">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+      <c r="H6" s="31">
+        <f t="shared" si="1"/>
+        <v>26.5</v>
+      </c>
+      <c r="I6" s="31">
+        <f t="shared" si="2"/>
+        <v>24.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="34"/>
+      <c r="B8" s="31"/>
+      <c r="D8" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" s="5">
+        <f>COUNT(E3:F3)</f>
+        <v>2</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="G8" s="16">
+        <f>AVERAGE(I3:I6)</f>
+        <v>9.375</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="I8" s="5">
+        <f>2^E8*(E9-1)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="34"/>
+      <c r="B9" s="31"/>
+      <c r="D9" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" s="5">
+        <v>2</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" s="5">
+        <f>SQRT(G8/(E9*2^(E8-2)))</f>
+        <v>2.1650635094610968</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="I9" s="5">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="34"/>
+      <c r="B10" s="31"/>
+    </row>
+    <row r="12" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="44"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="31"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="46"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="32"/>
+      <c r="F13" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="G13" s="5">
+        <f>1/(2*E9)*(G4+G6-G5-G3)</f>
+        <v>-2.75</v>
+      </c>
+      <c r="H13" s="5">
+        <f>$G$9</f>
+        <v>2.1650635094610968</v>
+      </c>
+      <c r="I13" s="5">
+        <f>G13/H13</f>
+        <v>-1.2701705922171767</v>
+      </c>
+      <c r="J13" s="5">
+        <f>_xlfn.T.DIST.2T(ABS(I13), $I$8)</f>
+        <v>0.27288073795194623</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="44"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="30"/>
+      <c r="F14" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G14" s="5">
+        <f>1/(2*E9)*(G5+G6-G4-G3)</f>
+        <v>10.75</v>
+      </c>
+      <c r="H14" s="5">
+        <f>$G$9</f>
+        <v>2.1650635094610968</v>
+      </c>
+      <c r="I14" s="5">
+        <f t="shared" ref="I14:I15" si="3">G14/H14</f>
+        <v>4.9652123150307812</v>
+      </c>
+      <c r="J14" s="5">
+        <f t="shared" ref="J14:J15" si="4">_xlfn.T.DIST.2T(ABS(I14), $I$8)</f>
+        <v>7.6775801621824036E-3</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F15" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="G15" s="6">
+        <f>1/(2*E9)*(G6+G3-G4-G5)</f>
+        <v>1.75</v>
+      </c>
+      <c r="H15" s="5">
+        <f>$G$9</f>
+        <v>2.1650635094610968</v>
+      </c>
+      <c r="I15" s="5">
+        <f t="shared" si="3"/>
+        <v>0.808290376865476</v>
+      </c>
+      <c r="J15" s="5">
+        <f t="shared" si="4"/>
+        <v>0.46425213971069967</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" s="1" customFormat="1" ht="50.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="35"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="36"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="17"/>
+    </row>
+    <row r="18" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="3"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="24"/>
+    </row>
+    <row r="20" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="G20" s="6">
+        <f>G14/2</f>
+        <v>5.375</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" s="6" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="34"/>
+      <c r="B22" s="33"/>
+      <c r="C22" s="5"/>
+      <c r="F22" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G22" s="65">
+        <f>AVERAGE(E3:F6)</f>
+        <v>21.625</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" s="6" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="34"/>
+      <c r="B23" s="33"/>
+      <c r="C23" s="5"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" spans="1:9" s="6" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="34"/>
+      <c r="B24" s="33"/>
+      <c r="C24" s="5"/>
+      <c r="F24" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G24" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="H24" s="5"/>
+    </row>
+    <row r="25" spans="1:9" s="6" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="34"/>
+      <c r="B25" s="33"/>
+      <c r="C25" s="5"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="5"/>
+    </row>
+    <row r="27" spans="1:9" s="6" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="47"/>
+      <c r="B27" s="47"/>
+      <c r="C27" s="48" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" s="48"/>
+      <c r="E27" s="48"/>
+      <c r="F27" s="48"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="5"/>
+    </row>
+    <row r="29" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E29" s="6">
+        <f>5.375*(-1)+22</f>
+        <v>16.625</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30" s="6">
+        <f>5.375*(1)+22</f>
+        <v>27.375</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E31" s="6">
+        <f>5.375*(-1)+22</f>
+        <v>16.625</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E32" s="40">
+        <v>27.375</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:F2"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>